<commit_message>
Add chassis fan thickness, header type, and daisy-chain fields.
</commit_message>
<xml_diff>
--- a/Datasheets/PcBuilder-Import-ChassisFans.xlsx
+++ b/Datasheets/PcBuilder-Import-ChassisFans.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,6 +441,26 @@
           <t>FansCountPerPack</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ThicknessMm</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>HeaderType</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>SupportsDaisyChain</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>MaxFansPerDaisyChain</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -461,6 +481,17 @@
       <c r="D2" t="n">
         <v>1</v>
       </c>
+      <c r="E2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -481,6 +512,17 @@
       <c r="D3" t="n">
         <v>1</v>
       </c>
+      <c r="E3" t="n">
+        <v>25</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -501,6 +543,17 @@
       <c r="D4" t="n">
         <v>1</v>
       </c>
+      <c r="E4" t="n">
+        <v>25</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -521,6 +574,17 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
+      <c r="E5" t="n">
+        <v>25</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -541,6 +605,17 @@
       <c r="D6" t="n">
         <v>1</v>
       </c>
+      <c r="E6" t="n">
+        <v>25</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -561,6 +636,17 @@
       <c r="D7" t="n">
         <v>3</v>
       </c>
+      <c r="E7" t="n">
+        <v>25</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -581,6 +667,17 @@
       <c r="D8" t="n">
         <v>3</v>
       </c>
+      <c r="E8" t="n">
+        <v>25</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G8" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -601,6 +698,17 @@
       <c r="D9" t="n">
         <v>3</v>
       </c>
+      <c r="E9" t="n">
+        <v>25</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G9" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -621,6 +729,17 @@
       <c r="D10" t="n">
         <v>3</v>
       </c>
+      <c r="E10" t="n">
+        <v>25</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G10" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -641,6 +760,17 @@
       <c r="D11" t="n">
         <v>3</v>
       </c>
+      <c r="E11" t="n">
+        <v>25</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G11" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -661,6 +791,17 @@
       <c r="D12" t="n">
         <v>1</v>
       </c>
+      <c r="E12" t="n">
+        <v>25</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G12" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -681,6 +822,17 @@
       <c r="D13" t="n">
         <v>1</v>
       </c>
+      <c r="E13" t="n">
+        <v>25</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G13" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -701,6 +853,17 @@
       <c r="D14" t="n">
         <v>3</v>
       </c>
+      <c r="E14" t="n">
+        <v>25</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G14" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -721,6 +884,17 @@
       <c r="D15" t="n">
         <v>3</v>
       </c>
+      <c r="E15" t="n">
+        <v>25</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G15" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -741,6 +915,17 @@
       <c r="D16" t="n">
         <v>3</v>
       </c>
+      <c r="E16" t="n">
+        <v>25</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G16" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -761,6 +946,17 @@
       <c r="D17" t="n">
         <v>2</v>
       </c>
+      <c r="E17" t="n">
+        <v>25</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G17" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -781,6 +977,17 @@
       <c r="D18" t="n">
         <v>2</v>
       </c>
+      <c r="E18" t="n">
+        <v>25</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G18" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -801,6 +1008,17 @@
       <c r="D19" t="n">
         <v>1</v>
       </c>
+      <c r="E19" t="n">
+        <v>25</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G19" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -821,6 +1039,17 @@
       <c r="D20" t="n">
         <v>3</v>
       </c>
+      <c r="E20" t="n">
+        <v>25</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G20" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -841,6 +1070,17 @@
       <c r="D21" t="n">
         <v>1</v>
       </c>
+      <c r="E21" t="n">
+        <v>25</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G21" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -861,6 +1101,17 @@
       <c r="D22" t="n">
         <v>1</v>
       </c>
+      <c r="E22" t="n">
+        <v>25</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G22" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -881,6 +1132,17 @@
       <c r="D23" t="n">
         <v>3</v>
       </c>
+      <c r="E23" t="n">
+        <v>25</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G23" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -901,6 +1163,17 @@
       <c r="D24" t="n">
         <v>1</v>
       </c>
+      <c r="E24" t="n">
+        <v>25</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G24" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -921,6 +1194,17 @@
       <c r="D25" t="n">
         <v>1</v>
       </c>
+      <c r="E25" t="n">
+        <v>25</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G25" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -941,6 +1225,17 @@
       <c r="D26" t="n">
         <v>3</v>
       </c>
+      <c r="E26" t="n">
+        <v>25</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G26" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -961,6 +1256,17 @@
       <c r="D27" t="n">
         <v>1</v>
       </c>
+      <c r="E27" t="n">
+        <v>25</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G27" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -981,6 +1287,17 @@
       <c r="D28" t="n">
         <v>1</v>
       </c>
+      <c r="E28" t="n">
+        <v>25</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G28" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1001,6 +1318,17 @@
       <c r="D29" t="n">
         <v>3</v>
       </c>
+      <c r="E29" t="n">
+        <v>25</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G29" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1020,6 +1348,17 @@
       </c>
       <c r="D30" t="n">
         <v>1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>25</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>FourPinPwm</t>
+        </is>
+      </c>
+      <c r="G30" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>